<commit_message>
Add updated Excel file for test automation
</commit_message>
<xml_diff>
--- a/Test_Automation/IT23181892.xlsx
+++ b/Test_Automation/IT23181892.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pinid\Documents\Github\IT23181892-ITPM-New_Assignment_01\Test_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAF433FF-0CDB-42AF-A9E2-559DB4CEA413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740B8A75-8B04-440E-9DA8-04BF1DCE1172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="208">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -52,6 +52,12 @@
     <t>මේක ප්‍රත්‍යක්ෂ කරගන්නේ කොහොමද?</t>
   </si>
   <si>
+    <t>මේක ප්රත්යක්ක්ෂා කරගන්නේ කොහොමද?</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
     <t>Neg_0002</t>
   </si>
   <si>
@@ -61,6 +67,9 @@
     <t>ඔයා ගම්‍යතා සංස්ථිති නියමය දන්නවද?</t>
   </si>
   <si>
+    <t>ඔයා ගම්යතා සංස්ථිති නියමය දන්නවද?</t>
+  </si>
+  <si>
     <t>Neg_0003</t>
   </si>
   <si>
@@ -73,6 +82,9 @@
     <t>තෘෂ්ණාව නසා දමන්න.</t>
   </si>
   <si>
+    <t>ත්රුෂ්ණාව නාසා දමන්න.</t>
+  </si>
+  <si>
     <t>Neg_0004</t>
   </si>
   <si>
@@ -82,6 +94,9 @@
     <t>සමචතුරස්‍ර හැඩේට එපා!</t>
   </si>
   <si>
+    <t>සමචතුරශ්ර හදේට එපා!</t>
+  </si>
+  <si>
     <t>Neg_0005</t>
   </si>
   <si>
@@ -91,6 +106,9 @@
     <t>ශ්‍රද්ධාවෙන් යුතුව පිළිගනිමු!</t>
   </si>
   <si>
+    <t>ශ්රද්ධාවෙන්‍යුතුව පිළිගනිමු!</t>
+  </si>
+  <si>
     <t>Neg_0006</t>
   </si>
   <si>
@@ -100,6 +118,9 @@
     <t>ප්‍රඥ්ඥාව වැඩෙන දිනයක් වේවා!</t>
   </si>
   <si>
+    <t>ප්රඥ්ඥාව වදෙන දිනයක් වේවා!</t>
+  </si>
+  <si>
     <t>Neg_0007</t>
   </si>
   <si>
@@ -109,6 +130,9 @@
     <t>මට ආධ්‍යාත්මික සහනය ඕනේ.</t>
   </si>
   <si>
+    <t>මට ආද්යාත්මික සහනය ඕනෑ.</t>
+  </si>
+  <si>
     <t>Neg_0008</t>
   </si>
   <si>
@@ -118,6 +142,9 @@
     <t>කරුණාකර ත්‍රිකෝණය අඳින්න.</t>
   </si>
   <si>
+    <t>කරුණාකර ත්රිකෝණය අදින්න.</t>
+  </si>
+  <si>
     <t>Neg_0009</t>
   </si>
   <si>
@@ -127,6 +154,9 @@
     <t>ඔව්, ඒක සම්පූර්ණ භ්‍රාන්තියක්.</t>
   </si>
   <si>
+    <t>ඔව්, ඒක සම්පූරණ භ්රාඅන්තියක්.</t>
+  </si>
+  <si>
     <t>Neg_0010</t>
   </si>
   <si>
@@ -136,6 +166,9 @@
     <t>මේ ගෙවෙන්නෙ සූර්‍ය සංක්‍රාණ්ති සමයක්!</t>
   </si>
   <si>
+    <t>මේ ගෙවෙන්නේ සූර්ය සංක්රාන්ති සමයක්!</t>
+  </si>
+  <si>
     <t>Neg_0011</t>
   </si>
   <si>
@@ -145,6 +178,9 @@
     <t>කිරි කිරි බෝලේ රැලි රැලි මාලේ</t>
   </si>
   <si>
+    <t>කිරි කිරි බොලේ රාලි රාලි මලේ</t>
+  </si>
+  <si>
     <t>Neg_0012</t>
   </si>
   <si>
@@ -154,6 +190,9 @@
     <t>සිලි සිලි සීතල ඇල්ලේ</t>
   </si>
   <si>
+    <t>සිලි සිලි සිතලා අල්ලේ</t>
+  </si>
+  <si>
     <t>Neg_0013</t>
   </si>
   <si>
@@ -163,6 +202,9 @@
     <t>අයියෝ... මේක මහා ව්‍යසනයක්!</t>
   </si>
   <si>
+    <t>අයියෝ... මේක මහා ව්යසනයක්!</t>
+  </si>
+  <si>
     <t>Neg_0014</t>
   </si>
   <si>
@@ -172,6 +214,9 @@
     <t>අපොයි ඒ ජෝතිශ්‍යවේදියා බොරුද කිව්වෙ?</t>
   </si>
   <si>
+    <t>අපොයිට් ඒ ජෝතිෂ්යවැඩියා බොරුද කිව්වේ?</t>
+  </si>
+  <si>
     <t>Neg_0015</t>
   </si>
   <si>
@@ -181,6 +226,9 @@
     <t>ප්ඥ්ඥාරතන හාමුදුරුවෝ</t>
   </si>
   <si>
+    <t>පඥ්ඥරටන හාමුදුරුවෝ</t>
+  </si>
+  <si>
     <t>Neg_0016</t>
   </si>
   <si>
@@ -190,6 +238,9 @@
     <t>ධර්මය අවබෝධ කරගන්න.</t>
   </si>
   <si>
+    <t>ධ්ර්මය අවබෝධ කරගන්න.</t>
+  </si>
+  <si>
     <t>Neg_0017</t>
   </si>
   <si>
@@ -199,6 +250,9 @@
     <t>අද shangri la එකේ buffet එකට යමුද?</t>
   </si>
   <si>
+    <t>අද ෂන්ග්රි ලා එකේ බුෆේට් එකට යමුද?</t>
+  </si>
+  <si>
     <t>Neg_0018</t>
   </si>
   <si>
@@ -208,6 +262,9 @@
     <t>උඹ නං පට්ට singer කෙනෙක්.</t>
   </si>
   <si>
+    <t>උඹ නම් පට්ට සින්ගර් කෙනෙක්.</t>
+  </si>
+  <si>
     <t>Neg_0019</t>
   </si>
   <si>
@@ -217,6 +274,9 @@
     <t>මේක under supervision යන්න ඕනෙ shipment එකක්.</t>
   </si>
   <si>
+    <t>මේක under supervision යන්න one shipment එකක්.</t>
+  </si>
+  <si>
     <t>Neg_0020</t>
   </si>
   <si>
@@ -226,6 +286,9 @@
     <t>මේ පාර kolkata knite riders cup එක උස්සයි වගේ</t>
   </si>
   <si>
+    <t>මේ පාර කොල්කටා ඤිටේ රිඩෙර්ස් කප් එක උස්සයි වගේ</t>
+  </si>
+  <si>
     <t>Neg_0021</t>
   </si>
   <si>
@@ -235,6 +298,9 @@
     <t>backend api එක වැඩ කරන්නෙ නෑ.</t>
   </si>
   <si>
+    <t>බක්එන්ඩ් අපි ඒක වැඩ කරන්නේ නෑ.</t>
+  </si>
+  <si>
     <t>Neg_0022</t>
   </si>
   <si>
@@ -244,6 +310,9 @@
     <t>මොනවද frontend එකට දාපු dependencies?</t>
   </si>
   <si>
+    <t>මොනවද ෆ්රොන්ට්එන්ඩ් එකට දාපු ඩෙපෙන්ඩෙන්සිස්?</t>
+  </si>
+  <si>
     <t>Neg_0023</t>
   </si>
   <si>
@@ -253,6 +322,9 @@
     <t>pixelssuite chat translator එක නං ජරාවක්.</t>
   </si>
   <si>
+    <t>පික්සෙල්ස්වීට් චාට් ට්රාන්ස්ලටර් එක නම් ජරාවක්.</t>
+  </si>
+  <si>
     <t>Neg_0024</t>
   </si>
   <si>
@@ -262,6 +334,9 @@
     <t>මගේ අලුත් song එක spotify දැම්මා.</t>
   </si>
   <si>
+    <t>මගේ අලුත් සොන්ග් එක ස්පොටිෆයි දැම්මා.</t>
+  </si>
+  <si>
     <t>Neg_0025</t>
   </si>
   <si>
@@ -271,6 +346,9 @@
     <t>O.T.P. එක ආවද?</t>
   </si>
   <si>
+    <t>ඕ.ට්.ප. ඒක ආවද?</t>
+  </si>
+  <si>
     <t>Neg_0026</t>
   </si>
   <si>
@@ -280,6 +358,9 @@
     <t>N.I.C. එකේවත් copy එකක් ගන්න.</t>
   </si>
   <si>
+    <t>න්.I.සී. ඒකෙවත් කොපි 1ක් ගන්න.</t>
+  </si>
+  <si>
     <t>Neg_0027</t>
   </si>
   <si>
@@ -289,6 +370,9 @@
     <t>lab එකේ equipments වැඩ කරන්නේ නෑ.</t>
   </si>
   <si>
+    <t>lab එකේ එච්පේන්ට්ස් වැඩ කරන්නේ නෑ.</t>
+  </si>
+  <si>
     <t>Neg_0028</t>
   </si>
   <si>
@@ -298,6 +382,9 @@
     <t>labs වලටම ගිහින් assignment 1ක දාමු</t>
   </si>
   <si>
+    <t>ලබ්ස් වලටම ගිහින් assignment එක දාමු.</t>
+  </si>
+  <si>
     <t>Neg_0029</t>
   </si>
   <si>
@@ -307,6 +394,9 @@
     <t>එයා ශ්‍රී ජයවර්ධනපුර කෝට්ටේ ඉන්නෙ.</t>
   </si>
   <si>
+    <t>එයා Sri Jayawardenepura Kotte ඉන්නේ.</t>
+  </si>
+  <si>
     <t>Neg_0030</t>
   </si>
   <si>
@@ -316,6 +406,9 @@
     <t>බත්තලංගුන්ඩුවේ ගිහින් තියනවද ඔයා?</t>
   </si>
   <si>
+    <t>බත්තලඟුඬුවෙ ගිහින් තියනවද ඔයා?</t>
+  </si>
+  <si>
     <t>Neg_0031</t>
   </si>
   <si>
@@ -325,6 +418,9 @@
     <t>john logie baird තමයි tv එක හොයාගත්තේ</t>
   </si>
   <si>
+    <t>ජොහ්න් ලෝගිඒ බෛර්ඩ් තමයි ටීවී එක හොයාගත්තෙ</t>
+  </si>
+  <si>
     <t>Neg_0032</t>
   </si>
   <si>
@@ -334,6 +430,9 @@
     <t>isaac newtonගෙ ඔලුවට වැටුනෙ මොකක්ද?</t>
   </si>
   <si>
+    <t>ඉසඅක් නැව්ටන්ගී ඔලුවට වැටුණේ මොකක්ද?</t>
+  </si>
+  <si>
     <t>Neg_0033</t>
   </si>
   <si>
@@ -343,6 +442,9 @@
     <t>භාගයක්(1/2)ක්ම මගේ එකෙන්ම කැපිලා.</t>
   </si>
   <si>
+    <t>බාගයක්(1/2කෑම මගේ 1න්ම කැපිලා.</t>
+  </si>
+  <si>
     <t>Neg_0034</t>
   </si>
   <si>
@@ -352,6 +454,9 @@
     <t>1st එකටත්(පළවෙනි) වඩා 100%ක්ම sure බං.</t>
   </si>
   <si>
+    <t>1st1(පලවෙනි)ටත්_වද_100%ක්ම_sure_bng.</t>
+  </si>
+  <si>
     <t>Neg_0035</t>
   </si>
   <si>
@@ -361,6 +466,9 @@
     <t>Rs. 1,500.99 cents වලටම බිල ඇවිත් නේද.</t>
   </si>
   <si>
+    <t>Rs.1,500.99centsltම_bila_awith_neda.</t>
+  </si>
+  <si>
     <t>Neg_0036</t>
   </si>
   <si>
@@ -370,6 +478,9 @@
     <t>$5ක්මයි ඉතුරු වුණේ.</t>
   </si>
   <si>
+    <t>5ක්මයි ඉතුරු වුණේ.</t>
+  </si>
+  <si>
     <t>Neg_0037</t>
   </si>
   <si>
@@ -379,6 +490,9 @@
     <t>24:00ටමයි වැඩේ පටන් ගන්නේ.</t>
   </si>
   <si>
+    <t>24:00 හර්ස් තමයි වැඩේ පටන් ගන්නේ.</t>
+  </si>
+  <si>
     <t>Neg_0038</t>
   </si>
   <si>
@@ -397,6 +511,9 @@
     <t>2026 Feb 29th එක දවසේම නිදා ගමු.</t>
   </si>
   <si>
+    <t>UI Error</t>
+  </si>
+  <si>
     <t>Neg_0040</t>
   </si>
   <si>
@@ -406,6 +523,9 @@
     <t>Feb 29වෙනිදා තමයි මගේ b'day එක.</t>
   </si>
   <si>
+    <t>පෙබරවාරි 29 වෙනිදා තමයි මගේ birthday එක.</t>
+  </si>
+  <si>
     <t>Neg_0041</t>
   </si>
   <si>
@@ -415,6 +535,9 @@
     <t>අපි knot 21ක වේගෙන් යනව සර්.</t>
   </si>
   <si>
+    <t>අපි කනොට් 21ක වේගෙන් යනවා sir.</t>
+  </si>
+  <si>
     <t>Neg_0042</t>
   </si>
   <si>
@@ -424,6 +547,9 @@
     <t>සූර්‍යාගෙ බාහිර උෂ්ණත්වය කෙල්වින් 5700ක් විතර.</t>
   </si>
   <si>
+    <t>සූර්යාගේ බාහිර උෂ්ණත්වය කැල්වින් 5700ක් විතර.</t>
+  </si>
+  <si>
     <t>Neg_0043</t>
   </si>
   <si>
@@ -433,6 +559,9 @@
     <t>translator එකක් හදාගන්න බැරිද බං උඹට? ඊයා.</t>
   </si>
   <si>
+    <t>ට්රාන්ස්ලටෝර් එකක් හදාගන්න බැරිද බං උබට? ඉයා.</t>
+  </si>
+  <si>
     <t>Neg_0044</t>
   </si>
   <si>
@@ -442,6 +571,9 @@
     <t>උඹට පුලුවන්ද මාව වාඩිකරන්න. පඹයා.</t>
   </si>
   <si>
+    <t>උබට පුලුවන්ද මාව වඩිකරන්න. පබාය.</t>
+  </si>
+  <si>
     <t>Neg_0045</t>
   </si>
   <si>
@@ -451,6 +583,9 @@
     <t>එයාගෙ insta id එක @nethmi_25</t>
   </si>
   <si>
+    <t>එයාගේ ඉන්ස්ටා ඉඩ් එක @නැත්නම්මි_25</t>
+  </si>
+  <si>
     <t>Neg_0046</t>
   </si>
   <si>
@@ -460,6 +595,9 @@
     <t>info-desk@vishwavidyalaya.lk එකට mail කරන්න.</t>
   </si>
   <si>
+    <t>info-desk@vishwavidyalaya.ලැක් එකට mail කරන්න.</t>
+  </si>
+  <si>
     <t>Neg_0047</t>
   </si>
   <si>
@@ -469,6 +607,9 @@
     <t>ඒකට නං මධුර කුලතුංගටත් හිනා😅💔</t>
   </si>
   <si>
+    <t>ඒකට නම් මධුර කුලතුංගටත් හිනා😅</t>
+  </si>
+  <si>
     <t>Neg_0048</t>
   </si>
   <si>
@@ -478,6 +619,9 @@
     <t>අද රෑ assignment deadline යකෝ🚨‼️</t>
   </si>
   <si>
+    <t>අද රෑ assignment deadline යකෝ!!️</t>
+  </si>
+  <si>
     <t>Neg_0049</t>
   </si>
   <si>
@@ -487,6 +631,9 @@
     <t>මෘත දේහය අඳුරගන්න පුලුවන්ද ඔයාට?</t>
   </si>
   <si>
+    <t>මෘදුත දේහය අදුරගන්න පුලුවන්ද ඔයාට?</t>
+  </si>
+  <si>
     <t>Neg_0050</t>
   </si>
   <si>
@@ -494,6 +641,9 @@
   </si>
   <si>
     <t>සංක්ෂේපන සඳහනය නිකන් කියවලා බලපන්.</t>
+  </si>
+  <si>
+    <t>සංක්ෂේපණ සන්ධාහනය නිකන් කියෝලා බලපන්.</t>
   </si>
 </sst>
 </file>
@@ -905,13 +1055,13 @@
     <col min="2" max="2" width="8.88671875" style="8" customWidth="1"/>
     <col min="3" max="3" width="22.109375" style="12" customWidth="1"/>
     <col min="4" max="4" width="25.33203125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.44140625" style="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" style="2" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" style="2" customWidth="1"/>
     <col min="8" max="8" width="16" style="2" customWidth="1"/>
     <col min="9" max="10" width="12.33203125" style="2" customWidth="1"/>
-    <col min="11" max="12" width="8.88671875" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="2"/>
+    <col min="11" max="13" width="8.88671875" style="2" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
@@ -947,791 +1097,990 @@
       <c r="D2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="4"/>
+      <c r="E2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="5"/>
+        <v>14</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="5"/>
+        <v>19</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="5"/>
+        <v>23</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="9"/>
-      <c r="F6" s="4"/>
+        <v>27</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="5"/>
+        <v>31</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="10"/>
-      <c r="F8" s="5"/>
+        <v>35</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="5"/>
+        <v>39</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="10"/>
-      <c r="F10" s="5"/>
+        <v>43</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="11" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E11" s="10"/>
-      <c r="F11" s="5"/>
+        <v>47</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="12" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="10"/>
-      <c r="F12" s="5"/>
+        <v>51</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="13" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="14" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="5"/>
+        <v>59</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="5"/>
+        <v>63</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="16" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="E16" s="10"/>
-      <c r="F16" s="5"/>
+        <v>67</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="17" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E17" s="10"/>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="F18" s="5"/>
+        <v>75</v>
+      </c>
+      <c r="E18" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="19" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E19" s="10"/>
-      <c r="F19" s="5"/>
+        <v>79</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="20" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E20" s="10"/>
-      <c r="F20" s="5"/>
+        <v>83</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="21" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="10"/>
-      <c r="F21" s="5"/>
+        <v>87</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="22" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="10"/>
-      <c r="F22" s="5"/>
+        <v>91</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="E23" s="10"/>
-      <c r="F23" s="5"/>
+        <v>95</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="24" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="5"/>
+        <v>99</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="25" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E25" s="10"/>
-      <c r="F25" s="5"/>
+        <v>103</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="E26" s="10"/>
-      <c r="F26" s="5"/>
+        <v>107</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="27" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="5"/>
+        <v>111</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="28" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>87</v>
+        <v>114</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="E28" s="10"/>
-      <c r="F28" s="5"/>
+        <v>115</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="29" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="E29" s="10"/>
-      <c r="F29" s="5"/>
+        <v>119</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="30" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>93</v>
+        <v>122</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="E30" s="10"/>
-      <c r="F30" s="5"/>
+        <v>123</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="E31" s="10"/>
-      <c r="F31" s="5"/>
+        <v>127</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="E32" s="10"/>
-      <c r="F32" s="5"/>
+        <v>131</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="33" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="E33" s="10"/>
-      <c r="F33" s="5"/>
+        <v>135</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="34" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="E34" s="10"/>
-      <c r="F34" s="5"/>
+        <v>139</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="35" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>107</v>
+        <v>141</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>108</v>
+        <v>142</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="E35" s="10"/>
-      <c r="F35" s="5"/>
+        <v>143</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="36" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>110</v>
+        <v>145</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="E36" s="10"/>
-      <c r="F36" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="37" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>114</v>
+        <v>150</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E37" s="10"/>
-      <c r="F37" s="5"/>
+        <v>151</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="38" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>116</v>
+        <v>153</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>117</v>
+        <v>154</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="E38" s="10"/>
-      <c r="F38" s="5"/>
+        <v>155</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="39" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>119</v>
+        <v>157</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>120</v>
+        <v>158</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="E39" s="10"/>
-      <c r="F39" s="5"/>
+        <v>159</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="40" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>122</v>
+        <v>160</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>123</v>
+        <v>161</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>124</v>
+        <v>162</v>
       </c>
       <c r="E40" s="10"/>
-      <c r="F40" s="5"/>
+      <c r="F40" s="5" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="41" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>126</v>
+        <v>165</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="E41" s="10"/>
-      <c r="F41" s="5"/>
+        <v>166</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="42" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>128</v>
+        <v>168</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="E42" s="10"/>
-      <c r="F42" s="5"/>
+        <v>170</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="43" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
-        <v>131</v>
+        <v>172</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>132</v>
+        <v>173</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="E43" s="10"/>
-      <c r="F43" s="5"/>
+        <v>174</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="44" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>134</v>
+        <v>176</v>
       </c>
       <c r="B44" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>135</v>
+        <v>177</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="E44" s="10"/>
-      <c r="F44" s="5"/>
+        <v>178</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="45" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="E45" s="10"/>
-      <c r="F45" s="5"/>
+        <v>182</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="46" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>140</v>
+        <v>184</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>141</v>
+        <v>185</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="E46" s="10"/>
-      <c r="F46" s="5"/>
+        <v>186</v>
+      </c>
+      <c r="E46" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="47" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
-        <v>143</v>
+        <v>188</v>
       </c>
       <c r="B47" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>144</v>
+        <v>189</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E47" s="10"/>
-      <c r="F47" s="5"/>
+        <v>190</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="48" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>146</v>
+        <v>192</v>
       </c>
       <c r="B48" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>147</v>
+        <v>193</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="E48" s="10"/>
-      <c r="F48" s="5"/>
+        <v>194</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="49" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
-        <v>149</v>
+        <v>196</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>150</v>
+        <v>197</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="E49" s="10"/>
-      <c r="F49" s="5"/>
+        <v>198</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="50" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>152</v>
+        <v>200</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C50" s="9" t="s">
-        <v>153</v>
+        <v>201</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="E50" s="10"/>
-      <c r="F50" s="5"/>
+        <v>202</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="51" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
       <c r="B51" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>156</v>
+        <v>205</v>
       </c>
       <c r="D51" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="E51" s="10"/>
-      <c r="F51" s="5"/>
+        <v>206</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added Types and evidence columns
</commit_message>
<xml_diff>
--- a/Test_Automation/IT23181892.xlsx
+++ b/Test_Automation/IT23181892.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pinid\Documents\Github\IT23181892-ITPM-New_Assignment_01\Test_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{740B8A75-8B04-440E-9DA8-04BF1DCE1172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC321A58-132B-49AB-9D12-930D6280876D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="298">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -644,13 +644,283 @@
   </si>
   <si>
     <t>සංක්ෂේපණ සන්ධාහනය නිකන් කියෝලා බලපන්.</t>
+  </si>
+  <si>
+    <t>Singlish input types covered</t>
+  </si>
+  <si>
+    <t>Evidence or rationale for the input type covered</t>
+  </si>
+  <si>
+    <t>Question forms</t>
+  </si>
+  <si>
+    <t>Command forms</t>
+  </si>
+  <si>
+    <t>Greetings</t>
+  </si>
+  <si>
+    <t>Requests</t>
+  </si>
+  <si>
+    <t>Response</t>
+  </si>
+  <si>
+    <t>General sentence</t>
+  </si>
+  <si>
+    <t>Repeated words</t>
+  </si>
+  <si>
+    <t>Input with punctuations</t>
+  </si>
+  <si>
+    <t>Question forms, punctuations</t>
+  </si>
+  <si>
+    <t>Personal Names</t>
+  </si>
+  <si>
+    <t>English phrases, Question forms</t>
+  </si>
+  <si>
+    <t>English word insertion, slang</t>
+  </si>
+  <si>
+    <t>Multi-word English phrases</t>
+  </si>
+  <si>
+    <t>Place names, English phrases</t>
+  </si>
+  <si>
+    <t>Digital terms</t>
+  </si>
+  <si>
+    <t>Digital terms, Question forms</t>
+  </si>
+  <si>
+    <t>Platform/app names</t>
+  </si>
+  <si>
+    <t>Acronyms, Question forms</t>
+  </si>
+  <si>
+    <t>Acronyms</t>
+  </si>
+  <si>
+    <t>English words, digital/technical</t>
+  </si>
+  <si>
+    <t>Numbers, English words</t>
+  </si>
+  <si>
+    <t>Place names</t>
+  </si>
+  <si>
+    <t>Place names, Question forms</t>
+  </si>
+  <si>
+    <t>Person names</t>
+  </si>
+  <si>
+    <t>Person names, Question forms</t>
+  </si>
+  <si>
+    <t>Numbers</t>
+  </si>
+  <si>
+    <t>Numbers, English words, slang</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Time formats</t>
+  </si>
+  <si>
+    <t>Time formats, Questions</t>
+  </si>
+  <si>
+    <t>Dates</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Slang, Question</t>
+  </si>
+  <si>
+    <t>Slang</t>
+  </si>
+  <si>
+    <t>Online identifiers</t>
+  </si>
+  <si>
+    <t>Emoji, Person names</t>
+  </si>
+  <si>
+    <t>Emoji, English words</t>
+  </si>
+  <si>
+    <t>Question form</t>
+  </si>
+  <si>
+    <t>suggestion/command</t>
+  </si>
+  <si>
+    <t>interrogative</t>
+  </si>
+  <si>
+    <t>urgency + emoji</t>
+  </si>
+  <si>
+    <t>emoji + name</t>
+  </si>
+  <si>
+    <t>emoji format</t>
+  </si>
+  <si>
+    <t>“@username”</t>
+  </si>
+  <si>
+    <t>insulting casual tone</t>
+  </si>
+  <si>
+    <t>“ban”, “ubata”</t>
+  </si>
+  <si>
+    <t>Kelvin measurement</t>
+  </si>
+  <si>
+    <t>“knot 21”</t>
+  </si>
+  <si>
+    <t>“Feb 29”</t>
+  </si>
+  <si>
+    <t>Full date</t>
+  </si>
+  <si>
+    <t>timestamp format</t>
+  </si>
+  <si>
+    <t>“24:00”</t>
+  </si>
+  <si>
+    <t>Dollar symbol</t>
+  </si>
+  <si>
+    <t>Rs. + decimal</t>
+  </si>
+  <si>
+    <t>“1st”, “100%”, “sure”</t>
+  </si>
+  <si>
+    <t>Fraction usage</t>
+  </si>
+  <si>
+    <t>Famous person</t>
+  </si>
+  <si>
+    <t>Scientist name</t>
+  </si>
+  <si>
+    <t>Location-based question</t>
+  </si>
+  <si>
+    <t>Sri Lankan city</t>
+  </si>
+  <si>
+    <t>“assignment 1ka”</t>
+  </si>
+  <si>
+    <t>“lab”, “equipments”</t>
+  </si>
+  <si>
+    <t>NIC</t>
+  </si>
+  <si>
+    <t>OTP format</t>
+  </si>
+  <si>
+    <t>"spotify"</t>
+  </si>
+  <si>
+    <t>App name mentioned</t>
+  </si>
+  <si>
+    <t>"frontend", "Dependencies"</t>
+  </si>
+  <si>
+    <t>"backend api"</t>
+  </si>
+  <si>
+    <t>“kolkata knight riders”</t>
+  </si>
+  <si>
+    <t>“under supervision”, “shipment”</t>
+  </si>
+  <si>
+    <t>“singer”, casual tone</t>
+  </si>
+  <si>
+    <t>“buffet”, “shangri la”</t>
+  </si>
+  <si>
+    <t>Instructional tone</t>
+  </si>
+  <si>
+    <t>Religious name</t>
+  </si>
+  <si>
+    <t>“?” + emotional tone</t>
+  </si>
+  <si>
+    <t>Ellipsis + exclamation</t>
+  </si>
+  <si>
+    <t>“sili sili” repetition</t>
+  </si>
+  <si>
+    <t>“kiri kiri”, “rali rali”</t>
+  </si>
+  <si>
+    <t>Informative statement</t>
+  </si>
+  <si>
+    <t>Starts with affirmation “ow”</t>
+  </si>
+  <si>
+    <t>“karunakara” polite request</t>
+  </si>
+  <si>
+    <t>Expression of need “one”</t>
+  </si>
+  <si>
+    <t>Blessing structure “wewa”</t>
+  </si>
+  <si>
+    <t>Formal welcoming tone</t>
+  </si>
+  <si>
+    <t>Negative command “epa!”</t>
+  </si>
+  <si>
+    <t>Imperative verb “damanna”</t>
+  </si>
+  <si>
+    <t>“dannawada?” → interrogative</t>
+  </si>
+  <si>
+    <t>Ends with “kohomadha?” indicating a question</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -683,6 +953,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.5"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -720,7 +997,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -767,6 +1044,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1048,7 +1334,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="49.95" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.88671875" style="2" customWidth="1"/>
@@ -1057,14 +1343,14 @@
     <col min="4" max="4" width="25.33203125" style="12" customWidth="1"/>
     <col min="5" max="5" width="44.44140625" style="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="16" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26.6640625" style="18" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="43.44140625" style="18" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="12.33203125" style="2" customWidth="1"/>
     <col min="11" max="13" width="8.88671875" style="2" customWidth="1"/>
     <col min="14" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1083,8 +1369,14 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G1" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -1103,8 +1395,14 @@
       <c r="F2" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G2" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
@@ -1123,8 +1421,14 @@
       <c r="F3" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G3" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
@@ -1143,8 +1447,14 @@
       <c r="F4" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G4" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>21</v>
       </c>
@@ -1163,8 +1473,14 @@
       <c r="F5" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G5" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>25</v>
       </c>
@@ -1183,8 +1499,14 @@
       <c r="F6" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G6" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>29</v>
       </c>
@@ -1203,8 +1525,14 @@
       <c r="F7" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G7" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>33</v>
       </c>
@@ -1223,8 +1551,14 @@
       <c r="F8" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G8" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>37</v>
       </c>
@@ -1243,8 +1577,14 @@
       <c r="F9" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G9" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>41</v>
       </c>
@@ -1263,8 +1603,14 @@
       <c r="F10" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G10" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>45</v>
       </c>
@@ -1283,8 +1629,14 @@
       <c r="F11" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G11" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
@@ -1303,8 +1655,14 @@
       <c r="F12" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G12" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>53</v>
       </c>
@@ -1323,8 +1681,14 @@
       <c r="F13" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G13" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>57</v>
       </c>
@@ -1343,8 +1707,14 @@
       <c r="F14" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G14" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>61</v>
       </c>
@@ -1363,8 +1733,14 @@
       <c r="F15" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G15" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>65</v>
       </c>
@@ -1383,8 +1759,14 @@
       <c r="F16" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G16" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>69</v>
       </c>
@@ -1403,8 +1785,14 @@
       <c r="F17" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G17" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>73</v>
       </c>
@@ -1417,14 +1805,20 @@
       <c r="D18" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="19" t="s">
         <v>76</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G18" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>77</v>
       </c>
@@ -1443,8 +1837,14 @@
       <c r="F19" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G19" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>81</v>
       </c>
@@ -1463,8 +1863,14 @@
       <c r="F20" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G20" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>85</v>
       </c>
@@ -1483,8 +1889,14 @@
       <c r="F21" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G21" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>89</v>
       </c>
@@ -1503,8 +1915,14 @@
       <c r="F22" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G22" s="10" t="s">
+        <v>224</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>93</v>
       </c>
@@ -1523,8 +1941,14 @@
       <c r="F23" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G23" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>97</v>
       </c>
@@ -1543,8 +1967,14 @@
       <c r="F24" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G24" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>101</v>
       </c>
@@ -1563,8 +1993,14 @@
       <c r="F25" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G25" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>105</v>
       </c>
@@ -1583,8 +2019,14 @@
       <c r="F26" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G26" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
         <v>109</v>
       </c>
@@ -1603,8 +2045,14 @@
       <c r="F27" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G27" s="10" t="s">
+        <v>228</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>113</v>
       </c>
@@ -1623,8 +2071,14 @@
       <c r="F28" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G28" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>117</v>
       </c>
@@ -1643,8 +2097,14 @@
       <c r="F29" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G29" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>121</v>
       </c>
@@ -1663,8 +2123,14 @@
       <c r="F30" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G30" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>125</v>
       </c>
@@ -1683,8 +2149,14 @@
       <c r="F31" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G31" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>129</v>
       </c>
@@ -1703,8 +2175,14 @@
       <c r="F32" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G32" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>133</v>
       </c>
@@ -1723,8 +2201,14 @@
       <c r="F33" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G33" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>137</v>
       </c>
@@ -1743,8 +2227,14 @@
       <c r="F34" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G34" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>141</v>
       </c>
@@ -1763,8 +2253,14 @@
       <c r="F35" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G35" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>145</v>
       </c>
@@ -1783,8 +2279,14 @@
       <c r="F36" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G36" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>149</v>
       </c>
@@ -1803,8 +2305,14 @@
       <c r="F37" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G37" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>153</v>
       </c>
@@ -1823,8 +2331,14 @@
       <c r="F38" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G38" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>157</v>
       </c>
@@ -1843,8 +2357,14 @@
       <c r="F39" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G39" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>160</v>
       </c>
@@ -1861,8 +2381,14 @@
       <c r="F40" s="5" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G40" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>164</v>
       </c>
@@ -1881,8 +2407,14 @@
       <c r="F41" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G41" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>168</v>
       </c>
@@ -1901,8 +2433,14 @@
       <c r="F42" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G42" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>172</v>
       </c>
@@ -1921,8 +2459,14 @@
       <c r="F43" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G43" s="10" t="s">
+        <v>241</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>176</v>
       </c>
@@ -1941,8 +2485,14 @@
       <c r="F44" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G44" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>180</v>
       </c>
@@ -1961,8 +2511,14 @@
       <c r="F45" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G45" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>184</v>
       </c>
@@ -1981,8 +2537,14 @@
       <c r="F46" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G46" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
         <v>188</v>
       </c>
@@ -2001,8 +2563,14 @@
       <c r="F47" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G47" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>192</v>
       </c>
@@ -2021,8 +2589,14 @@
       <c r="F48" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G48" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="5" t="s">
         <v>196</v>
       </c>
@@ -2041,8 +2615,14 @@
       <c r="F49" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G49" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="H49" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>200</v>
       </c>
@@ -2061,8 +2641,14 @@
       <c r="F50" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G50" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
         <v>204</v>
       </c>
@@ -2080,6 +2666,12 @@
       </c>
       <c r="F51" s="5" t="s">
         <v>11</v>
+      </c>
+      <c r="G51" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>